<commit_message>
basic per capita graph
</commit_message>
<xml_diff>
--- a/GDP-per-capita.xlsx
+++ b/GDP-per-capita.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chris\Dropbox\RMIT work\Teaching\Economics of AI\Content\economic-growth-projection\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA6D8824-E811-4B1C-BCF1-447407D5F9C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3382292-C8B8-44F7-8DD5-8078235F9674}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{0CAB2825-0D3D-40D2-9155-B23B4180D9EF}"/>
   </bookViews>
@@ -121,8 +121,8 @@
     <numFmt numFmtId="164" formatCode="mmm\-yyyy"/>
     <numFmt numFmtId="165" formatCode="0.0;\-0.0;0.0;@"/>
     <numFmt numFmtId="166" formatCode="0;\-0;0;@"/>
-    <numFmt numFmtId="175" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="177" formatCode="_-&quot;$&quot;* #,##0_-;\-&quot;$&quot;* #,##0_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="167" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="168" formatCode="_-&quot;$&quot;* #,##0_-;\-&quot;$&quot;* #,##0_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -201,9 +201,9 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="175" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" indent="2"/>
     </xf>
   </cellXfs>
@@ -2620,9 +2620,8 @@
       <c r="E2" t="str">
         <f>"{ quarter: """ &amp; A2 &amp; """, " &amp;
  "annualized_gdp_million: " &amp; TEXT(B2,"0") &amp; ", " &amp;
- "population_persons: " &amp; TEXT(C2,"0") &amp; ", " &amp;
- "annualized_gdp_pc: " &amp; TEXT(D2,"0") &amp; " },"</f>
-        <v>{ quarter: "Quarter date", annualized_gdp_million: GDP millions, population_persons: Population, annualized_gdp_pc: Per capita },</v>
+ "population_persons: " &amp; TEXT(C2,"0") &amp; "},"</f>
+        <v>{ quarter: "Quarter date", annualized_gdp_million: GDP millions, population_persons: Population},</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -2643,11 +2642,10 @@
         <v>49742.617249535957</v>
       </c>
       <c r="E3" t="str">
-        <f t="shared" ref="E3:E66" si="0">"{ quarter: """ &amp; A3 &amp; """, " &amp;
+        <f>"{ quarter: """ &amp; A3 &amp; """, " &amp;
  "annualized_gdp_million: " &amp; TEXT(B3,"0") &amp; ", " &amp;
- "population_persons: " &amp; TEXT(C3,"0") &amp; ", " &amp;
- "annualized_gdp_pc: " &amp; TEXT(D3,"0") &amp; " },"</f>
-        <v>{ quarter: "1981-Q2", annualized_gdp_million: 742324, population_persons: 14923300, annualized_gdp_pc: 49743 },</v>
+ "population_persons: " &amp; TEXT(C3,"0") &amp; "},"</f>
+        <v>{ quarter: "1981-Q2", annualized_gdp_million: 742324, population_persons: 14923300},</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -2664,12 +2662,14 @@
         <v>14988700</v>
       </c>
       <c r="D4" s="16">
-        <f t="shared" ref="D4:D67" si="1">(B4*1000000)/C4</f>
+        <f t="shared" ref="D4:D67" si="0">(B4*1000000)/C4</f>
         <v>50524.728628900441</v>
       </c>
       <c r="E4" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1981-Q3", annualized_gdp_million: 757300, population_persons: 14988700, annualized_gdp_pc: 50525 },</v>
+        <f t="shared" ref="E4:E67" si="1">"{ quarter: """ &amp; A4 &amp; """, " &amp;
+ "annualized_gdp_million: " &amp; TEXT(B4,"0") &amp; ", " &amp;
+ "population_persons: " &amp; TEXT(C4,"0") &amp; "},"</f>
+        <v>{ quarter: "1981-Q3", annualized_gdp_million: 757300, population_persons: 14988700},</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
@@ -2686,12 +2686,12 @@
         <v>15054100</v>
       </c>
       <c r="D5" s="16">
+        <f t="shared" si="0"/>
+        <v>50098.245660650588</v>
+      </c>
+      <c r="E5" t="str">
         <f t="shared" si="1"/>
-        <v>50098.245660650588</v>
-      </c>
-      <c r="E5" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1981-Q4", annualized_gdp_million: 754184, population_persons: 15054100, annualized_gdp_pc: 50098 },</v>
+        <v>{ quarter: "1981-Q4", annualized_gdp_million: 754184, population_persons: 15054100},</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
@@ -2708,12 +2708,12 @@
         <v>15121700</v>
       </c>
       <c r="D6" s="16">
+        <f t="shared" si="0"/>
+        <v>49476.183233366617</v>
+      </c>
+      <c r="E6" t="str">
         <f t="shared" si="1"/>
-        <v>49476.183233366617</v>
-      </c>
-      <c r="E6" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1982-Q1", annualized_gdp_million: 748164, population_persons: 15121700, annualized_gdp_pc: 49476 },</v>
+        <v>{ quarter: "1982-Q1", annualized_gdp_million: 748164, population_persons: 15121700},</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
@@ -2730,12 +2730,12 @@
         <v>15184200</v>
       </c>
       <c r="D7" s="16">
+        <f t="shared" si="0"/>
+        <v>49709.829954821456</v>
+      </c>
+      <c r="E7" t="str">
         <f t="shared" si="1"/>
-        <v>49709.829954821456</v>
-      </c>
-      <c r="E7" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1982-Q2", annualized_gdp_million: 754804, population_persons: 15184200, annualized_gdp_pc: 49710 },</v>
+        <v>{ quarter: "1982-Q2", annualized_gdp_million: 754804, population_persons: 15184200},</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
@@ -2752,12 +2752,12 @@
         <v>15239300</v>
       </c>
       <c r="D8" s="16">
+        <f t="shared" si="0"/>
+        <v>49203.309863313931</v>
+      </c>
+      <c r="E8" t="str">
         <f t="shared" si="1"/>
-        <v>49203.309863313931</v>
-      </c>
-      <c r="E8" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1982-Q3", annualized_gdp_million: 749824, population_persons: 15239300, annualized_gdp_pc: 49203 },</v>
+        <v>{ quarter: "1982-Q3", annualized_gdp_million: 749824, population_persons: 15239300},</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
@@ -2774,12 +2774,12 @@
         <v>15288900</v>
       </c>
       <c r="D9" s="16">
+        <f t="shared" si="0"/>
+        <v>48254.616094028999</v>
+      </c>
+      <c r="E9" t="str">
         <f t="shared" si="1"/>
-        <v>48254.616094028999</v>
-      </c>
-      <c r="E9" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1982-Q4", annualized_gdp_million: 737760, population_persons: 15288900, annualized_gdp_pc: 48255 },</v>
+        <v>{ quarter: "1982-Q4", annualized_gdp_million: 737760, population_persons: 15288900},</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
@@ -2796,12 +2796,12 @@
         <v>15346200</v>
       </c>
       <c r="D10" s="16">
+        <f t="shared" si="0"/>
+        <v>47611.525980372993</v>
+      </c>
+      <c r="E10" t="str">
         <f t="shared" si="1"/>
-        <v>47611.525980372993</v>
-      </c>
-      <c r="E10" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1983-Q1", annualized_gdp_million: 730656, population_persons: 15346200, annualized_gdp_pc: 47612 },</v>
+        <v>{ quarter: "1983-Q1", annualized_gdp_million: 730656, population_persons: 15346200},</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
@@ -2818,12 +2818,12 @@
         <v>15393500</v>
       </c>
       <c r="D11" s="16">
+        <f t="shared" si="0"/>
+        <v>47368.04495403904</v>
+      </c>
+      <c r="E11" t="str">
         <f t="shared" si="1"/>
-        <v>47368.04495403904</v>
-      </c>
-      <c r="E11" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1983-Q2", annualized_gdp_million: 729160, population_persons: 15393500, annualized_gdp_pc: 47368 },</v>
+        <v>{ quarter: "1983-Q2", annualized_gdp_million: 729160, population_persons: 15393500},</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
@@ -2840,12 +2840,12 @@
         <v>15439000</v>
       </c>
       <c r="D12" s="16">
+        <f t="shared" si="0"/>
+        <v>48552.367381307078</v>
+      </c>
+      <c r="E12" t="str">
         <f t="shared" si="1"/>
-        <v>48552.367381307078</v>
-      </c>
-      <c r="E12" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1983-Q3", annualized_gdp_million: 749600, population_persons: 15439000, annualized_gdp_pc: 48552 },</v>
+        <v>{ quarter: "1983-Q3", annualized_gdp_million: 749600, population_persons: 15439000},</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
@@ -2862,12 +2862,12 @@
         <v>15483500</v>
       </c>
       <c r="D13" s="16">
+        <f t="shared" si="0"/>
+        <v>49230.471146704556</v>
+      </c>
+      <c r="E13" t="str">
         <f t="shared" si="1"/>
-        <v>49230.471146704556</v>
-      </c>
-      <c r="E13" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1983-Q4", annualized_gdp_million: 762260, population_persons: 15483500, annualized_gdp_pc: 49230 },</v>
+        <v>{ quarter: "1983-Q4", annualized_gdp_million: 762260, population_persons: 15483500},</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
@@ -2884,12 +2884,12 @@
         <v>15531500</v>
       </c>
       <c r="D14" s="16">
+        <f t="shared" si="0"/>
+        <v>50278.981424846279</v>
+      </c>
+      <c r="E14" t="str">
         <f t="shared" si="1"/>
-        <v>50278.981424846279</v>
-      </c>
-      <c r="E14" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1984-Q1", annualized_gdp_million: 780908, population_persons: 15531500, annualized_gdp_pc: 50279 },</v>
+        <v>{ quarter: "1984-Q1", annualized_gdp_million: 780908, population_persons: 15531500},</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
@@ -2906,12 +2906,12 @@
         <v>15579400</v>
       </c>
       <c r="D15" s="16">
+        <f t="shared" si="0"/>
+        <v>50710.040181265002</v>
+      </c>
+      <c r="E15" t="str">
         <f t="shared" si="1"/>
-        <v>50710.040181265002</v>
-      </c>
-      <c r="E15" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1984-Q2", annualized_gdp_million: 790032, population_persons: 15579400, annualized_gdp_pc: 50710 },</v>
+        <v>{ quarter: "1984-Q2", annualized_gdp_million: 790032, population_persons: 15579400},</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
@@ -2928,12 +2928,12 @@
         <v>15628500</v>
       </c>
       <c r="D16" s="16">
+        <f t="shared" si="0"/>
+        <v>51016.028409636245</v>
+      </c>
+      <c r="E16" t="str">
         <f t="shared" si="1"/>
-        <v>51016.028409636245</v>
-      </c>
-      <c r="E16" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1984-Q3", annualized_gdp_million: 797304, population_persons: 15628500, annualized_gdp_pc: 51016 },</v>
+        <v>{ quarter: "1984-Q3", annualized_gdp_million: 797304, population_persons: 15628500},</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
@@ -2950,12 +2950,12 @@
         <v>15677300</v>
       </c>
       <c r="D17" s="16">
+        <f t="shared" si="0"/>
+        <v>51164.167299216067</v>
+      </c>
+      <c r="E17" t="str">
         <f t="shared" si="1"/>
-        <v>51164.167299216067</v>
-      </c>
-      <c r="E17" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1984-Q4", annualized_gdp_million: 802116, population_persons: 15677300, annualized_gdp_pc: 51164 },</v>
+        <v>{ quarter: "1984-Q4", annualized_gdp_million: 802116, population_persons: 15677300},</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
@@ -2972,12 +2972,12 @@
         <v>15736700</v>
       </c>
       <c r="D18" s="16">
+        <f t="shared" si="0"/>
+        <v>51723.169406546484</v>
+      </c>
+      <c r="E18" t="str">
         <f t="shared" si="1"/>
-        <v>51723.169406546484</v>
-      </c>
-      <c r="E18" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1985-Q1", annualized_gdp_million: 813952, population_persons: 15736700, annualized_gdp_pc: 51723 },</v>
+        <v>{ quarter: "1985-Q1", annualized_gdp_million: 813952, population_persons: 15736700},</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
@@ -2994,12 +2994,12 @@
         <v>15788300</v>
       </c>
       <c r="D19" s="16">
+        <f t="shared" si="0"/>
+        <v>52706.624525756415</v>
+      </c>
+      <c r="E19" t="str">
         <f t="shared" si="1"/>
-        <v>52706.624525756415</v>
-      </c>
-      <c r="E19" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1985-Q2", annualized_gdp_million: 832148, population_persons: 15788300, annualized_gdp_pc: 52707 },</v>
+        <v>{ quarter: "1985-Q2", annualized_gdp_million: 832148, population_persons: 15788300},</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
@@ -3016,12 +3016,12 @@
         <v>15839700</v>
       </c>
       <c r="D20" s="16">
+        <f t="shared" si="0"/>
+        <v>53209.088555970127</v>
+      </c>
+      <c r="E20" t="str">
         <f t="shared" si="1"/>
-        <v>53209.088555970127</v>
-      </c>
-      <c r="E20" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1985-Q3", annualized_gdp_million: 842816, population_persons: 15839700, annualized_gdp_pc: 53209 },</v>
+        <v>{ quarter: "1985-Q3", annualized_gdp_million: 842816, population_persons: 15839700},</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
@@ -3038,12 +3038,12 @@
         <v>15900600</v>
       </c>
       <c r="D21" s="16">
+        <f t="shared" si="0"/>
+        <v>52857.124888368991</v>
+      </c>
+      <c r="E21" t="str">
         <f t="shared" si="1"/>
-        <v>52857.124888368991</v>
-      </c>
-      <c r="E21" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1985-Q4", annualized_gdp_million: 840460, population_persons: 15900600, annualized_gdp_pc: 52857 },</v>
+        <v>{ quarter: "1985-Q4", annualized_gdp_million: 840460, population_persons: 15900600},</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
@@ -3060,12 +3060,12 @@
         <v>15961500</v>
       </c>
       <c r="D22" s="16">
+        <f t="shared" si="0"/>
+        <v>53018.325345362275</v>
+      </c>
+      <c r="E22" t="str">
         <f t="shared" si="1"/>
-        <v>53018.325345362275</v>
-      </c>
-      <c r="E22" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1986-Q1", annualized_gdp_million: 846252, population_persons: 15961500, annualized_gdp_pc: 53018 },</v>
+        <v>{ quarter: "1986-Q1", annualized_gdp_million: 846252, population_persons: 15961500},</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
@@ -3082,12 +3082,12 @@
         <v>16018400</v>
       </c>
       <c r="D23" s="16">
+        <f t="shared" si="0"/>
+        <v>52734.355491185139</v>
+      </c>
+      <c r="E23" t="str">
         <f t="shared" si="1"/>
-        <v>52734.355491185139</v>
-      </c>
-      <c r="E23" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1986-Q2", annualized_gdp_million: 844720, population_persons: 16018400, annualized_gdp_pc: 52734 },</v>
+        <v>{ quarter: "1986-Q2", annualized_gdp_million: 844720, population_persons: 16018400},</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
@@ -3104,12 +3104,12 @@
         <v>16075000</v>
       </c>
       <c r="D24" s="16">
+        <f t="shared" si="0"/>
+        <v>52687.029548989114</v>
+      </c>
+      <c r="E24" t="str">
         <f t="shared" si="1"/>
-        <v>52687.029548989114</v>
-      </c>
-      <c r="E24" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1986-Q3", annualized_gdp_million: 846944, population_persons: 16075000, annualized_gdp_pc: 52687 },</v>
+        <v>{ quarter: "1986-Q3", annualized_gdp_million: 846944, population_persons: 16075000},</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
@@ -3126,12 +3126,12 @@
         <v>16138800</v>
       </c>
       <c r="D25" s="16">
+        <f t="shared" si="0"/>
+        <v>53344.238729025703</v>
+      </c>
+      <c r="E25" t="str">
         <f t="shared" si="1"/>
-        <v>53344.238729025703</v>
-      </c>
-      <c r="E25" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1986-Q4", annualized_gdp_million: 860912, population_persons: 16138800, annualized_gdp_pc: 53344 },</v>
+        <v>{ quarter: "1986-Q4", annualized_gdp_million: 860912, population_persons: 16138800},</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
@@ -3148,12 +3148,12 @@
         <v>16204000</v>
       </c>
       <c r="D26" s="16">
+        <f t="shared" si="0"/>
+        <v>53656.381140459147</v>
+      </c>
+      <c r="E26" t="str">
         <f t="shared" si="1"/>
-        <v>53656.381140459147</v>
-      </c>
-      <c r="E26" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1987-Q1", annualized_gdp_million: 869448, population_persons: 16204000, annualized_gdp_pc: 53656 },</v>
+        <v>{ quarter: "1987-Q1", annualized_gdp_million: 869448, population_persons: 16204000},</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
@@ -3170,12 +3170,12 @@
         <v>16263900</v>
       </c>
       <c r="D27" s="16">
+        <f t="shared" si="0"/>
+        <v>54311.20456962967</v>
+      </c>
+      <c r="E27" t="str">
         <f t="shared" si="1"/>
-        <v>54311.20456962967</v>
-      </c>
-      <c r="E27" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1987-Q2", annualized_gdp_million: 883312, population_persons: 16263900, annualized_gdp_pc: 54311 },</v>
+        <v>{ quarter: "1987-Q2", annualized_gdp_million: 883312, population_persons: 16263900},</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
@@ -3192,12 +3192,12 @@
         <v>16328900</v>
       </c>
       <c r="D28" s="16">
+        <f t="shared" si="0"/>
+        <v>55069.478041999158</v>
+      </c>
+      <c r="E28" t="str">
         <f t="shared" si="1"/>
-        <v>55069.478041999158</v>
-      </c>
-      <c r="E28" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1987-Q3", annualized_gdp_million: 899224, population_persons: 16328900, annualized_gdp_pc: 55069 },</v>
+        <v>{ quarter: "1987-Q3", annualized_gdp_million: 899224, population_persons: 16328900},</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
@@ -3214,12 +3214,12 @@
         <v>16394599.999999998</v>
       </c>
       <c r="D29" s="16">
+        <f t="shared" si="0"/>
+        <v>55958.425335171341</v>
+      </c>
+      <c r="E29" t="str">
         <f t="shared" si="1"/>
-        <v>55958.425335171341</v>
-      </c>
-      <c r="E29" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1987-Q4", annualized_gdp_million: 917416, population_persons: 16394600, annualized_gdp_pc: 55958 },</v>
+        <v>{ quarter: "1987-Q4", annualized_gdp_million: 917416, population_persons: 16394600},</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
@@ -3236,12 +3236,12 @@
         <v>16471800</v>
       </c>
       <c r="D30" s="16">
+        <f t="shared" si="0"/>
+        <v>55923.457059944878</v>
+      </c>
+      <c r="E30" t="str">
         <f t="shared" si="1"/>
-        <v>55923.457059944878</v>
-      </c>
-      <c r="E30" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1988-Q1", annualized_gdp_million: 921160, population_persons: 16471800, annualized_gdp_pc: 55923 },</v>
+        <v>{ quarter: "1988-Q1", annualized_gdp_million: 921160, population_persons: 16471800},</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
@@ -3258,12 +3258,12 @@
         <v>16532200</v>
       </c>
       <c r="D31" s="16">
+        <f t="shared" si="0"/>
+        <v>55774.307109761554</v>
+      </c>
+      <c r="E31" t="str">
         <f t="shared" si="1"/>
-        <v>55774.307109761554</v>
-      </c>
-      <c r="E31" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1988-Q2", annualized_gdp_million: 922072, population_persons: 16532200, annualized_gdp_pc: 55774 },</v>
+        <v>{ quarter: "1988-Q2", annualized_gdp_million: 922072, population_persons: 16532200},</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
@@ -3280,12 +3280,12 @@
         <v>16612599.999999998</v>
       </c>
       <c r="D32" s="16">
+        <f t="shared" si="0"/>
+        <v>55948.376533474599</v>
+      </c>
+      <c r="E32" t="str">
         <f t="shared" si="1"/>
-        <v>55948.376533474599</v>
-      </c>
-      <c r="E32" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1988-Q3", annualized_gdp_million: 929448, population_persons: 16612600, annualized_gdp_pc: 55948 },</v>
+        <v>{ quarter: "1988-Q3", annualized_gdp_million: 929448, population_persons: 16612600},</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
@@ -3302,12 +3302,12 @@
         <v>16687099.999999998</v>
       </c>
       <c r="D33" s="16">
+        <f t="shared" si="0"/>
+        <v>56606.12089578178</v>
+      </c>
+      <c r="E33" t="str">
         <f t="shared" si="1"/>
-        <v>56606.12089578178</v>
-      </c>
-      <c r="E33" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1988-Q4", annualized_gdp_million: 944592, population_persons: 16687100, annualized_gdp_pc: 56606 },</v>
+        <v>{ quarter: "1988-Q4", annualized_gdp_million: 944592, population_persons: 16687100},</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
@@ -3324,12 +3324,12 @@
         <v>16764000</v>
       </c>
       <c r="D34" s="16">
+        <f t="shared" si="0"/>
+        <v>56872.584108804578</v>
+      </c>
+      <c r="E34" t="str">
         <f t="shared" si="1"/>
-        <v>56872.584108804578</v>
-      </c>
-      <c r="E34" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1989-Q1", annualized_gdp_million: 953412, population_persons: 16764000, annualized_gdp_pc: 56873 },</v>
+        <v>{ quarter: "1989-Q1", annualized_gdp_million: 953412, population_persons: 16764000},</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
@@ -3346,12 +3346,12 @@
         <v>16814400</v>
       </c>
       <c r="D35" s="16">
+        <f t="shared" si="0"/>
+        <v>57937.006375487676</v>
+      </c>
+      <c r="E35" t="str">
         <f t="shared" si="1"/>
-        <v>57937.006375487676</v>
-      </c>
-      <c r="E35" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1989-Q2", annualized_gdp_million: 974176, population_persons: 16814400, annualized_gdp_pc: 57937 },</v>
+        <v>{ quarter: "1989-Q2", annualized_gdp_million: 974176, population_persons: 16814400},</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
@@ -3368,12 +3368,12 @@
         <v>16872000</v>
       </c>
       <c r="D36" s="16">
+        <f t="shared" si="0"/>
+        <v>58221.431958274065</v>
+      </c>
+      <c r="E36" t="str">
         <f t="shared" si="1"/>
-        <v>58221.431958274065</v>
-      </c>
-      <c r="E36" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1989-Q3", annualized_gdp_million: 982312, population_persons: 16872000, annualized_gdp_pc: 58221 },</v>
+        <v>{ quarter: "1989-Q3", annualized_gdp_million: 982312, population_persons: 16872000},</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
@@ -3390,12 +3390,12 @@
         <v>16936700</v>
       </c>
       <c r="D37" s="16">
+        <f t="shared" si="0"/>
+        <v>57838.894235594889</v>
+      </c>
+      <c r="E37" t="str">
         <f t="shared" si="1"/>
-        <v>57838.894235594889</v>
-      </c>
-      <c r="E37" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1989-Q4", annualized_gdp_million: 979600, population_persons: 16936700, annualized_gdp_pc: 57839 },</v>
+        <v>{ quarter: "1989-Q4", annualized_gdp_million: 979600, population_persons: 16936700},</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
@@ -3412,12 +3412,12 @@
         <v>17005600</v>
       </c>
       <c r="D38" s="16">
+        <f t="shared" si="0"/>
+        <v>58049.818883191416</v>
+      </c>
+      <c r="E38" t="str">
         <f t="shared" si="1"/>
-        <v>58049.818883191416</v>
-      </c>
-      <c r="E38" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1990-Q1", annualized_gdp_million: 987172, population_persons: 17005600, annualized_gdp_pc: 58050 },</v>
+        <v>{ quarter: "1990-Q1", annualized_gdp_million: 987172, population_persons: 17005600},</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
@@ -3434,12 +3434,12 @@
         <v>17065100</v>
       </c>
       <c r="D39" s="16">
+        <f t="shared" si="0"/>
+        <v>57928.05198914744</v>
+      </c>
+      <c r="E39" t="str">
         <f t="shared" si="1"/>
-        <v>57928.05198914744</v>
-      </c>
-      <c r="E39" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1990-Q2", annualized_gdp_million: 988548, population_persons: 17065100, annualized_gdp_pc: 57928 },</v>
+        <v>{ quarter: "1990-Q2", annualized_gdp_million: 988548, population_persons: 17065100},</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
@@ -3456,12 +3456,12 @@
         <v>17121100</v>
       </c>
       <c r="D40" s="16">
+        <f t="shared" si="0"/>
+        <v>57428.085812243371</v>
+      </c>
+      <c r="E40" t="str">
         <f t="shared" si="1"/>
-        <v>57428.085812243371</v>
-      </c>
-      <c r="E40" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1990-Q3", annualized_gdp_million: 983232, population_persons: 17121100, annualized_gdp_pc: 57428 },</v>
+        <v>{ quarter: "1990-Q3", annualized_gdp_million: 983232, population_persons: 17121100},</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
@@ -3478,12 +3478,12 @@
         <v>17169800</v>
       </c>
       <c r="D41" s="16">
+        <f t="shared" si="0"/>
+        <v>57580.868734638723</v>
+      </c>
+      <c r="E41" t="str">
         <f t="shared" si="1"/>
-        <v>57580.868734638723</v>
-      </c>
-      <c r="E41" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1990-Q4", annualized_gdp_million: 988652, population_persons: 17169800, annualized_gdp_pc: 57581 },</v>
+        <v>{ quarter: "1990-Q4", annualized_gdp_million: 988652, population_persons: 17169800},</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
@@ -3500,12 +3500,12 @@
         <v>17237400</v>
       </c>
       <c r="D42" s="16">
+        <f t="shared" si="0"/>
+        <v>56634.295195331084</v>
+      </c>
+      <c r="E42" t="str">
         <f t="shared" si="1"/>
-        <v>56634.295195331084</v>
-      </c>
-      <c r="E42" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1991-Q1", annualized_gdp_million: 976228, population_persons: 17237400, annualized_gdp_pc: 56634 },</v>
+        <v>{ quarter: "1991-Q1", annualized_gdp_million: 976228, population_persons: 17237400},</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
@@ -3522,12 +3522,12 @@
         <v>17284000</v>
       </c>
       <c r="D43" s="16">
+        <f t="shared" si="0"/>
+        <v>56379.773200648</v>
+      </c>
+      <c r="E43" t="str">
         <f t="shared" si="1"/>
-        <v>56379.773200648</v>
-      </c>
-      <c r="E43" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1991-Q2", annualized_gdp_million: 974468, population_persons: 17284000, annualized_gdp_pc: 56380 },</v>
+        <v>{ quarter: "1991-Q2", annualized_gdp_million: 974468, population_persons: 17284000},</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.35">
@@ -3544,12 +3544,12 @@
         <v>17338900</v>
       </c>
       <c r="D44" s="16">
+        <f t="shared" si="0"/>
+        <v>56447.640853802724</v>
+      </c>
+      <c r="E44" t="str">
         <f t="shared" si="1"/>
-        <v>56447.640853802724</v>
-      </c>
-      <c r="E44" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1991-Q3", annualized_gdp_million: 978740, population_persons: 17338900, annualized_gdp_pc: 56448 },</v>
+        <v>{ quarter: "1991-Q3", annualized_gdp_million: 978740, population_persons: 17338900},</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.35">
@@ -3566,12 +3566,12 @@
         <v>17379000</v>
       </c>
       <c r="D45" s="16">
+        <f t="shared" si="0"/>
+        <v>56355.601588123594</v>
+      </c>
+      <c r="E45" t="str">
         <f t="shared" si="1"/>
-        <v>56355.601588123594</v>
-      </c>
-      <c r="E45" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1991-Q4", annualized_gdp_million: 979404, population_persons: 17379000, annualized_gdp_pc: 56356 },</v>
+        <v>{ quarter: "1991-Q4", annualized_gdp_million: 979404, population_persons: 17379000},</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.35">
@@ -3592,8 +3592,8 @@
         <v>56591.423804418249</v>
       </c>
       <c r="E46" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1992-Q1", annualized_gdp_million: 987028, population_persons: 17441300, annualized_gdp_pc: 56591 },</v>
+        <f t="shared" si="1"/>
+        <v>{ quarter: "1992-Q1", annualized_gdp_million: 987028, population_persons: 17441300},</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
@@ -3610,12 +3610,12 @@
         <v>17478600</v>
       </c>
       <c r="D47" s="16">
+        <f t="shared" si="0"/>
+        <v>56881.214742599521</v>
+      </c>
+      <c r="E47" t="str">
         <f t="shared" si="1"/>
-        <v>56881.214742599521</v>
-      </c>
-      <c r="E47" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1992-Q2", annualized_gdp_million: 994204, population_persons: 17478600, annualized_gdp_pc: 56881 },</v>
+        <v>{ quarter: "1992-Q2", annualized_gdp_million: 994204, population_persons: 17478600},</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.35">
@@ -3632,12 +3632,12 @@
         <v>17523300</v>
       </c>
       <c r="D48" s="16">
+        <f t="shared" si="0"/>
+        <v>57295.372446970607</v>
+      </c>
+      <c r="E48" t="str">
         <f t="shared" si="1"/>
-        <v>57295.372446970607</v>
-      </c>
-      <c r="E48" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1992-Q3", annualized_gdp_million: 1004004, population_persons: 17523300, annualized_gdp_pc: 57295 },</v>
+        <v>{ quarter: "1992-Q3", annualized_gdp_million: 1004004, population_persons: 17523300},</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.35">
@@ -3654,12 +3654,12 @@
         <v>17557100</v>
       </c>
       <c r="D49" s="16">
+        <f t="shared" si="0"/>
+        <v>58374.788547083517</v>
+      </c>
+      <c r="E49" t="str">
         <f t="shared" si="1"/>
-        <v>58374.788547083517</v>
-      </c>
-      <c r="E49" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1992-Q4", annualized_gdp_million: 1024892, population_persons: 17557100, annualized_gdp_pc: 58375 },</v>
+        <v>{ quarter: "1992-Q4", annualized_gdp_million: 1024892, population_persons: 17557100},</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.35">
@@ -3676,12 +3676,12 @@
         <v>17609600</v>
       </c>
       <c r="D50" s="16">
+        <f t="shared" si="0"/>
+        <v>58603.034708340907</v>
+      </c>
+      <c r="E50" t="str">
         <f t="shared" si="1"/>
-        <v>58603.034708340907</v>
-      </c>
-      <c r="E50" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1993-Q1", annualized_gdp_million: 1031976, population_persons: 17609600, annualized_gdp_pc: 58603 },</v>
+        <v>{ quarter: "1993-Q1", annualized_gdp_million: 1031976, population_persons: 17609600},</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.35">
@@ -3698,12 +3698,12 @@
         <v>17634800</v>
       </c>
       <c r="D51" s="16">
+        <f t="shared" si="0"/>
+        <v>58856.579036904302</v>
+      </c>
+      <c r="E51" t="str">
         <f t="shared" si="1"/>
-        <v>58856.579036904302</v>
-      </c>
-      <c r="E51" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1993-Q2", annualized_gdp_million: 1037924, population_persons: 17634800, annualized_gdp_pc: 58857 },</v>
+        <v>{ quarter: "1993-Q2", annualized_gdp_million: 1037924, population_persons: 17634800},</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.35">
@@ -3720,12 +3720,12 @@
         <v>17683700</v>
       </c>
       <c r="D52" s="16">
+        <f t="shared" si="0"/>
+        <v>58769.148990313115</v>
+      </c>
+      <c r="E52" t="str">
         <f t="shared" si="1"/>
-        <v>58769.148990313115</v>
-      </c>
-      <c r="E52" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1993-Q3", annualized_gdp_million: 1039256, population_persons: 17683700, annualized_gdp_pc: 58769 },</v>
+        <v>{ quarter: "1993-Q3", annualized_gdp_million: 1039256, population_persons: 17683700},</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.35">
@@ -3742,12 +3742,12 @@
         <v>17719100</v>
       </c>
       <c r="D53" s="16">
+        <f t="shared" si="0"/>
+        <v>59721.994909447996</v>
+      </c>
+      <c r="E53" t="str">
         <f t="shared" si="1"/>
-        <v>59721.994909447996</v>
-      </c>
-      <c r="E53" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1993-Q4", annualized_gdp_million: 1058220, population_persons: 17719100, annualized_gdp_pc: 59722 },</v>
+        <v>{ quarter: "1993-Q4", annualized_gdp_million: 1058220, population_persons: 17719100},</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.35">
@@ -3764,12 +3764,12 @@
         <v>17772100</v>
       </c>
       <c r="D54" s="16">
+        <f t="shared" si="0"/>
+        <v>60534.208112715998</v>
+      </c>
+      <c r="E54" t="str">
         <f t="shared" si="1"/>
-        <v>60534.208112715998</v>
-      </c>
-      <c r="E54" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1994-Q1", annualized_gdp_million: 1075820, population_persons: 17772100, annualized_gdp_pc: 60534 },</v>
+        <v>{ quarter: "1994-Q1", annualized_gdp_million: 1075820, population_persons: 17772100},</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.35">
@@ -3786,12 +3786,12 @@
         <v>17805500</v>
       </c>
       <c r="D55" s="16">
+        <f t="shared" si="0"/>
+        <v>61141.332734267504</v>
+      </c>
+      <c r="E55" t="str">
         <f t="shared" si="1"/>
-        <v>61141.332734267504</v>
-      </c>
-      <c r="E55" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1994-Q2", annualized_gdp_million: 1088652, population_persons: 17805500, annualized_gdp_pc: 61141 },</v>
+        <v>{ quarter: "1994-Q2", annualized_gdp_million: 1088652, population_persons: 17805500},</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.35">
@@ -3808,12 +3808,12 @@
         <v>17859300</v>
       </c>
       <c r="D56" s="16">
+        <f t="shared" si="0"/>
+        <v>61419.428533033213</v>
+      </c>
+      <c r="E56" t="str">
         <f t="shared" si="1"/>
-        <v>61419.428533033213</v>
-      </c>
-      <c r="E56" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1994-Q3", annualized_gdp_million: 1096908, population_persons: 17859300, annualized_gdp_pc: 61419 },</v>
+        <v>{ quarter: "1994-Q3", annualized_gdp_million: 1096908, population_persons: 17859300},</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.35">
@@ -3830,12 +3830,12 @@
         <v>17893400</v>
       </c>
       <c r="D57" s="16">
+        <f t="shared" si="0"/>
+        <v>61985.536566555267</v>
+      </c>
+      <c r="E57" t="str">
         <f t="shared" si="1"/>
-        <v>61985.536566555267</v>
-      </c>
-      <c r="E57" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1994-Q4", annualized_gdp_million: 1109132, population_persons: 17893400, annualized_gdp_pc: 61986 },</v>
+        <v>{ quarter: "1994-Q4", annualized_gdp_million: 1109132, population_persons: 17893400},</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.35">
@@ -3852,12 +3852,12 @@
         <v>17951600</v>
       </c>
       <c r="D58" s="16">
+        <f t="shared" si="0"/>
+        <v>61731.544820517389</v>
+      </c>
+      <c r="E58" t="str">
         <f t="shared" si="1"/>
-        <v>61731.544820517389</v>
-      </c>
-      <c r="E58" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1995-Q1", annualized_gdp_million: 1108180, population_persons: 17951600, annualized_gdp_pc: 61732 },</v>
+        <v>{ quarter: "1995-Q1", annualized_gdp_million: 1108180, population_persons: 17951600},</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.35">
@@ -3874,12 +3874,12 @@
         <v>18004900</v>
       </c>
       <c r="D59" s="16">
+        <f t="shared" si="0"/>
+        <v>61835.389255147209</v>
+      </c>
+      <c r="E59" t="str">
         <f t="shared" si="1"/>
-        <v>61835.389255147209</v>
-      </c>
-      <c r="E59" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1995-Q2", annualized_gdp_million: 1113340, population_persons: 18004900, annualized_gdp_pc: 61835 },</v>
+        <v>{ quarter: "1995-Q2", annualized_gdp_million: 1113340, population_persons: 18004900},</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.35">
@@ -3896,12 +3896,12 @@
         <v>18062200</v>
       </c>
       <c r="D60" s="16">
+        <f t="shared" si="0"/>
+        <v>63064.742943827441</v>
+      </c>
+      <c r="E60" t="str">
         <f t="shared" si="1"/>
-        <v>63064.742943827441</v>
-      </c>
-      <c r="E60" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1995-Q3", annualized_gdp_million: 1139088, population_persons: 18062200, annualized_gdp_pc: 63065 },</v>
+        <v>{ quarter: "1995-Q3", annualized_gdp_million: 1139088, population_persons: 18062200},</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.35">
@@ -3918,12 +3918,12 @@
         <v>18119600</v>
       </c>
       <c r="D61" s="16">
+        <f t="shared" si="0"/>
+        <v>62853.926135234775</v>
+      </c>
+      <c r="E61" t="str">
         <f t="shared" si="1"/>
-        <v>62853.926135234775</v>
-      </c>
-      <c r="E61" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1995-Q4", annualized_gdp_million: 1138888, population_persons: 18119600, annualized_gdp_pc: 62854 },</v>
+        <v>{ quarter: "1995-Q4", annualized_gdp_million: 1138888, population_persons: 18119600},</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.35">
@@ -3940,12 +3940,12 @@
         <v>18176000</v>
       </c>
       <c r="D62" s="16">
+        <f t="shared" si="0"/>
+        <v>63636.00352112676</v>
+      </c>
+      <c r="E62" t="str">
         <f t="shared" si="1"/>
-        <v>63636.00352112676</v>
-      </c>
-      <c r="E62" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1996-Q1", annualized_gdp_million: 1156648, population_persons: 18176000, annualized_gdp_pc: 63636 },</v>
+        <v>{ quarter: "1996-Q1", annualized_gdp_million: 1156648, population_persons: 18176000},</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.35">
@@ -3962,12 +3962,12 @@
         <v>18224800</v>
       </c>
       <c r="D63" s="16">
+        <f t="shared" si="0"/>
+        <v>63869.672095167029</v>
+      </c>
+      <c r="E63" t="str">
         <f t="shared" si="1"/>
-        <v>63869.672095167029</v>
-      </c>
-      <c r="E63" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1996-Q2", annualized_gdp_million: 1164012, population_persons: 18224800, annualized_gdp_pc: 63870 },</v>
+        <v>{ quarter: "1996-Q2", annualized_gdp_million: 1164012, population_persons: 18224800},</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.35">
@@ -3984,12 +3984,12 @@
         <v>18281300</v>
       </c>
       <c r="D64" s="16">
+        <f t="shared" si="0"/>
+        <v>64175.523622499495</v>
+      </c>
+      <c r="E64" t="str">
         <f t="shared" si="1"/>
-        <v>64175.523622499495</v>
-      </c>
-      <c r="E64" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1996-Q3", annualized_gdp_million: 1173212, population_persons: 18281300, annualized_gdp_pc: 64176 },</v>
+        <v>{ quarter: "1996-Q3", annualized_gdp_million: 1173212, population_persons: 18281300},</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.35">
@@ -4006,12 +4006,12 @@
         <v>18330100</v>
       </c>
       <c r="D65" s="16">
+        <f t="shared" si="0"/>
+        <v>64613.286343227803</v>
+      </c>
+      <c r="E65" t="str">
         <f t="shared" si="1"/>
-        <v>64613.286343227803</v>
-      </c>
-      <c r="E65" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1996-Q4", annualized_gdp_million: 1184368, population_persons: 18330100, annualized_gdp_pc: 64613 },</v>
+        <v>{ quarter: "1996-Q4", annualized_gdp_million: 1184368, population_persons: 18330100},</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.35">
@@ -4028,12 +4028,12 @@
         <v>18388700</v>
       </c>
       <c r="D66" s="16">
+        <f t="shared" si="0"/>
+        <v>64856.351998781858</v>
+      </c>
+      <c r="E66" t="str">
         <f t="shared" si="1"/>
-        <v>64856.351998781858</v>
-      </c>
-      <c r="E66" t="str">
-        <f t="shared" si="0"/>
-        <v>{ quarter: "1997-Q1", annualized_gdp_million: 1192624, population_persons: 18388700, annualized_gdp_pc: 64856 },</v>
+        <v>{ quarter: "1997-Q1", annualized_gdp_million: 1192624, population_persons: 18388700},</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.35">
@@ -4050,15 +4050,12 @@
         <v>18423000</v>
       </c>
       <c r="D67" s="16">
+        <f t="shared" si="0"/>
+        <v>66676.871302176631</v>
+      </c>
+      <c r="E67" t="str">
         <f t="shared" si="1"/>
-        <v>66676.871302176631</v>
-      </c>
-      <c r="E67" t="str">
-        <f t="shared" ref="E67:E83" si="2">"{ quarter: """ &amp; A67 &amp; """, " &amp;
- "annualized_gdp_million: " &amp; TEXT(B67,"0") &amp; ", " &amp;
- "population_persons: " &amp; TEXT(C67,"0") &amp; ", " &amp;
- "annualized_gdp_pc: " &amp; TEXT(D67,"0") &amp; " },"</f>
-        <v>{ quarter: "1997-Q2", annualized_gdp_million: 1228388, population_persons: 18423000, annualized_gdp_pc: 66677 },</v>
+        <v>{ quarter: "1997-Q2", annualized_gdp_million: 1228388, population_persons: 18423000},</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.35">
@@ -4075,12 +4072,14 @@
         <v>18468700</v>
       </c>
       <c r="D68" s="16">
-        <f t="shared" ref="D68:D77" si="3">(B68*1000000)/C68</f>
+        <f t="shared" ref="D68:D77" si="2">(B68*1000000)/C68</f>
         <v>66604.363057497278</v>
       </c>
       <c r="E68" t="str">
-        <f t="shared" si="2"/>
-        <v>{ quarter: "1997-Q3", annualized_gdp_million: 1230096, population_persons: 18468700, annualized_gdp_pc: 66604 },</v>
+        <f t="shared" ref="E68:E131" si="3">"{ quarter: """ &amp; A68 &amp; """, " &amp;
+ "annualized_gdp_million: " &amp; TEXT(B68,"0") &amp; ", " &amp;
+ "population_persons: " &amp; TEXT(C68,"0") &amp; "},"</f>
+        <v>{ quarter: "1997-Q3", annualized_gdp_million: 1230096, population_persons: 18468700},</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.35">
@@ -4097,12 +4096,12 @@
         <v>18510000</v>
       </c>
       <c r="D69" s="16">
+        <f t="shared" si="2"/>
+        <v>67402.485143165861</v>
+      </c>
+      <c r="E69" t="str">
         <f t="shared" si="3"/>
-        <v>67402.485143165861</v>
-      </c>
-      <c r="E69" t="str">
-        <f t="shared" si="2"/>
-        <v>{ quarter: "1997-Q4", annualized_gdp_million: 1247620, population_persons: 18510000, annualized_gdp_pc: 67402 },</v>
+        <v>{ quarter: "1997-Q4", annualized_gdp_million: 1247620, population_persons: 18510000},</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.35">
@@ -4119,12 +4118,12 @@
         <v>18572400</v>
       </c>
       <c r="D70" s="16">
+        <f t="shared" si="2"/>
+        <v>67596.002670629532</v>
+      </c>
+      <c r="E70" t="str">
         <f t="shared" si="3"/>
-        <v>67596.002670629532</v>
-      </c>
-      <c r="E70" t="str">
-        <f t="shared" si="2"/>
-        <v>{ quarter: "1998-Q1", annualized_gdp_million: 1255420, population_persons: 18572400, annualized_gdp_pc: 67596 },</v>
+        <v>{ quarter: "1998-Q1", annualized_gdp_million: 1255420, population_persons: 18572400},</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.35">
@@ -4141,12 +4140,12 @@
         <v>18607600</v>
       </c>
       <c r="D71" s="16">
+        <f t="shared" si="2"/>
+        <v>68159.891657172338</v>
+      </c>
+      <c r="E71" t="str">
         <f t="shared" si="3"/>
-        <v>68159.891657172338</v>
-      </c>
-      <c r="E71" t="str">
-        <f t="shared" si="2"/>
-        <v>{ quarter: "1998-Q2", annualized_gdp_million: 1268292, population_persons: 18607600, annualized_gdp_pc: 68160 },</v>
+        <v>{ quarter: "1998-Q2", annualized_gdp_million: 1268292, population_persons: 18607600},</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.35">
@@ -4163,12 +4162,12 @@
         <v>18658400</v>
       </c>
       <c r="D72" s="16">
+        <f t="shared" si="2"/>
+        <v>69238.734296617069</v>
+      </c>
+      <c r="E72" t="str">
         <f t="shared" si="3"/>
-        <v>69238.734296617069</v>
-      </c>
-      <c r="E72" t="str">
-        <f t="shared" si="2"/>
-        <v>{ quarter: "1998-Q3", annualized_gdp_million: 1291884, population_persons: 18658400, annualized_gdp_pc: 69239 },</v>
+        <v>{ quarter: "1998-Q3", annualized_gdp_million: 1291884, population_persons: 18658400},</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.35">
@@ -4185,12 +4184,12 @@
         <v>18705600</v>
       </c>
       <c r="D73" s="16">
+        <f t="shared" si="2"/>
+        <v>70137.28509109572</v>
+      </c>
+      <c r="E73" t="str">
         <f t="shared" si="3"/>
-        <v>70137.28509109572</v>
-      </c>
-      <c r="E73" t="str">
-        <f t="shared" si="2"/>
-        <v>{ quarter: "1998-Q4", annualized_gdp_million: 1311960, population_persons: 18705600, annualized_gdp_pc: 70137 },</v>
+        <v>{ quarter: "1998-Q4", annualized_gdp_million: 1311960, population_persons: 18705600},</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.35">
@@ -4207,12 +4206,12 @@
         <v>18770500</v>
       </c>
       <c r="D74" s="16">
+        <f t="shared" si="2"/>
+        <v>70419.221650994907</v>
+      </c>
+      <c r="E74" t="str">
         <f t="shared" si="3"/>
-        <v>70419.221650994907</v>
-      </c>
-      <c r="E74" t="str">
-        <f t="shared" si="2"/>
-        <v>{ quarter: "1999-Q1", annualized_gdp_million: 1321804, population_persons: 18770500, annualized_gdp_pc: 70419 },</v>
+        <v>{ quarter: "1999-Q1", annualized_gdp_million: 1321804, population_persons: 18770500},</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.35">
@@ -4229,12 +4228,12 @@
         <v>18812300</v>
       </c>
       <c r="D75" s="16">
+        <f t="shared" si="2"/>
+        <v>70551.500879743573</v>
+      </c>
+      <c r="E75" t="str">
         <f t="shared" si="3"/>
-        <v>70551.500879743573</v>
-      </c>
-      <c r="E75" t="str">
-        <f t="shared" si="2"/>
-        <v>{ quarter: "1999-Q2", annualized_gdp_million: 1327236, population_persons: 18812300, annualized_gdp_pc: 70552 },</v>
+        <v>{ quarter: "1999-Q2", annualized_gdp_million: 1327236, population_persons: 18812300},</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.35">
@@ -4251,12 +4250,12 @@
         <v>18867700</v>
       </c>
       <c r="D76" s="16">
+        <f t="shared" si="2"/>
+        <v>71100.558096641354</v>
+      </c>
+      <c r="E76" t="str">
         <f t="shared" si="3"/>
-        <v>71100.558096641354</v>
-      </c>
-      <c r="E76" t="str">
-        <f t="shared" si="2"/>
-        <v>{ quarter: "1999-Q3", annualized_gdp_million: 1341504, population_persons: 18867700, annualized_gdp_pc: 71101 },</v>
+        <v>{ quarter: "1999-Q3", annualized_gdp_million: 1341504, population_persons: 18867700},</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.35">
@@ -4273,12 +4272,12 @@
         <v>18919200</v>
       </c>
       <c r="D77" s="16">
+        <f t="shared" si="2"/>
+        <v>72123.557021438537</v>
+      </c>
+      <c r="E77" t="str">
         <f t="shared" si="3"/>
-        <v>72123.557021438537</v>
-      </c>
-      <c r="E77" t="str">
-        <f t="shared" si="2"/>
-        <v>{ quarter: "1999-Q4", annualized_gdp_million: 1364520, population_persons: 18919200, annualized_gdp_pc: 72124 },</v>
+        <v>{ quarter: "1999-Q4", annualized_gdp_million: 1364520, population_persons: 18919200},</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.35">
@@ -4299,8 +4298,8 @@
         <v>72140.81435952535</v>
       </c>
       <c r="E78" t="str">
-        <f t="shared" si="2"/>
-        <v>{ quarter: "2000-Q1", annualized_gdp_million: 1369716, population_persons: 18986700, annualized_gdp_pc: 72141 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2000-Q1", annualized_gdp_million: 1369716, population_persons: 18986700},</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.35">
@@ -4321,8 +4320,8 @@
         <v>72686.664424451359</v>
       </c>
       <c r="E79" t="str">
-        <f t="shared" si="2"/>
-        <v>{ quarter: "2000-Q2", annualized_gdp_million: 1383140, population_persons: 19028800, annualized_gdp_pc: 72687 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2000-Q2", annualized_gdp_million: 1383140, population_persons: 19028800},</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.35">
@@ -4343,8 +4342,8 @@
         <v>72653.672849208844</v>
       </c>
       <c r="E80" t="str">
-        <f t="shared" si="2"/>
-        <v>{ quarter: "2000-Q3", annualized_gdp_million: 1386668, population_persons: 19086000, annualized_gdp_pc: 72654 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2000-Q3", annualized_gdp_million: 1386668, population_persons: 19086000},</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.35">
@@ -4365,8 +4364,8 @@
         <v>72173.867614022252</v>
       </c>
       <c r="E81" t="str">
-        <f t="shared" si="2"/>
-        <v>{ quarter: "2000-Q4", annualized_gdp_million: 1381480, population_persons: 19141000, annualized_gdp_pc: 72174 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2000-Q4", annualized_gdp_million: 1381480, population_persons: 19141000},</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.35">
@@ -4387,8 +4386,8 @@
         <v>72529.180450658518</v>
       </c>
       <c r="E82" t="str">
-        <f t="shared" si="2"/>
-        <v>{ quarter: "2001-Q1", annualized_gdp_million: 1394388, population_persons: 19225200, annualized_gdp_pc: 72529 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2001-Q1", annualized_gdp_million: 1394388, population_persons: 19225200},</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.35">
@@ -4409,8 +4408,8 @@
         <v>72991.641893259046</v>
       </c>
       <c r="E83" t="str">
-        <f t="shared" si="2"/>
-        <v>{ quarter: "2001-Q2", annualized_gdp_million: 1406892, population_persons: 19274700, annualized_gdp_pc: 72992 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2001-Q2", annualized_gdp_million: 1406892, population_persons: 19274700},</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.35">
@@ -4431,11 +4430,8 @@
         <v>73633.019643956519</v>
       </c>
       <c r="E84" t="str">
-        <f>"{ quarter: """ &amp; A84 &amp; """, " &amp;
- "annualized_gdp_million: " &amp; TEXT(B84,"0") &amp; ", " &amp;
- "population_persons: " &amp; TEXT(C84,"0") &amp; ", " &amp;
- "annualized_gdp_pc: " &amp; TEXT(D84,"0") &amp; " },"</f>
-        <v>{ quarter: "2001-Q3", annualized_gdp_million: 1423260, population_persons: 19329100, annualized_gdp_pc: 73633 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2001-Q3", annualized_gdp_million: 1423260, population_persons: 19329100},</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.35">
@@ -4456,11 +4452,8 @@
         <v>74281.381373636294</v>
       </c>
       <c r="E85" t="str">
-        <f t="shared" ref="E85:E121" si="5">"{ quarter: """ &amp; A85 &amp; """, " &amp;
- "annualized_gdp_million: " &amp; TEXT(B85,"0") &amp; ", " &amp;
- "population_persons: " &amp; TEXT(C85,"0") &amp; ", " &amp;
- "annualized_gdp_pc: " &amp; TEXT(D85,"0") &amp; " },"</f>
-        <v>{ quarter: "2001-Q4", annualized_gdp_million: 1440056, population_persons: 19386500, annualized_gdp_pc: 74281 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2001-Q4", annualized_gdp_million: 1440056, population_persons: 19386500},</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.35">
@@ -4481,8 +4474,8 @@
         <v>74609.065767423686</v>
       </c>
       <c r="E86" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2002-Q1", annualized_gdp_million: 1451400, population_persons: 19453400, annualized_gdp_pc: 74609 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2002-Q1", annualized_gdp_million: 1451400, population_persons: 19453400},</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.35">
@@ -4503,8 +4496,8 @@
         <v>75728.999958964254</v>
       </c>
       <c r="E87" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2002-Q2", annualized_gdp_million: 1476352, population_persons: 19495200, annualized_gdp_pc: 75729 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2002-Q2", annualized_gdp_million: 1476352, population_persons: 19495200},</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.35">
@@ -4525,8 +4518,8 @@
         <v>75706.356879415209</v>
       </c>
       <c r="E88" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2002-Q3", annualized_gdp_million: 1479976, population_persons: 19548900, annualized_gdp_pc: 75706 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2002-Q3", annualized_gdp_million: 1479976, population_persons: 19548900},</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.35">
@@ -4547,8 +4540,8 @@
         <v>76125.149193589517</v>
       </c>
       <c r="E89" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2002-Q4", annualized_gdp_million: 1492464, population_persons: 19605400, annualized_gdp_pc: 76125 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2002-Q4", annualized_gdp_million: 1492464, population_persons: 19605400},</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.35">
@@ -4569,8 +4562,8 @@
         <v>76017.604667473046</v>
       </c>
       <c r="E90" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2003-Q1", annualized_gdp_million: 1495768, population_persons: 19676600, annualized_gdp_pc: 76018 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2003-Q1", annualized_gdp_million: 1495768, population_persons: 19676600},</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.35">
@@ -4591,8 +4584,8 @@
         <v>76155.714553743019</v>
       </c>
       <c r="E91" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2003-Q2", annualized_gdp_million: 1501844, population_persons: 19720700, annualized_gdp_pc: 76156 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2003-Q2", annualized_gdp_million: 1501844, population_persons: 19720700},</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.35">
@@ -4613,8 +4606,8 @@
         <v>77240.33297257933</v>
       </c>
       <c r="E92" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2003-Q3", annualized_gdp_million: 1527304, population_persons: 19773400, annualized_gdp_pc: 77240 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2003-Q3", annualized_gdp_million: 1527304, population_persons: 19773400},</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.35">
@@ -4635,8 +4628,8 @@
         <v>78336.628469980627</v>
       </c>
       <c r="E93" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2003-Q4", annualized_gdp_million: 1553196, population_persons: 19827200, annualized_gdp_pc: 78337 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2003-Q4", annualized_gdp_million: 1553196, population_persons: 19827200},</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.35">
@@ -4657,8 +4650,8 @@
         <v>78668.549972102279</v>
       </c>
       <c r="E94" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2004-Q1", annualized_gdp_million: 1565040, population_persons: 19894100, annualized_gdp_pc: 78669 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2004-Q1", annualized_gdp_million: 1565040, population_persons: 19894100},</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.35">
@@ -4679,8 +4672,8 @@
         <v>79101.576805952034</v>
       </c>
       <c r="E95" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2004-Q2", annualized_gdp_million: 1576708, population_persons: 19932700, annualized_gdp_pc: 79102 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2004-Q2", annualized_gdp_million: 1576708, population_persons: 19932700},</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.35">
@@ -4701,8 +4694,8 @@
         <v>79396.889398039988</v>
       </c>
       <c r="E96" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2004-Q3", annualized_gdp_million: 1587120, population_persons: 19989700, annualized_gdp_pc: 79397 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2004-Q3", annualized_gdp_million: 1587120, population_persons: 19989700},</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.35">
@@ -4723,8 +4716,8 @@
         <v>79779.706674648303</v>
       </c>
       <c r="E97" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2004-Q4", annualized_gdp_million: 1599264, population_persons: 20046000, annualized_gdp_pc: 79780 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2004-Q4", annualized_gdp_million: 1599264, population_persons: 20046000},</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.35">
@@ -4745,8 +4738,8 @@
         <v>80116.065306609162</v>
       </c>
       <c r="E98" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2005-Q1", annualized_gdp_million: 1612464, population_persons: 20126600, annualized_gdp_pc: 80116 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2005-Q1", annualized_gdp_million: 1612464, population_persons: 20126600},</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.35">
@@ -4767,8 +4760,8 @@
         <v>80273.185044209196</v>
       </c>
       <c r="E99" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2005-Q2", annualized_gdp_million: 1619656, population_persons: 20176800, annualized_gdp_pc: 80273 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2005-Q2", annualized_gdp_million: 1619656, population_persons: 20176800},</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.35">
@@ -4789,8 +4782,8 @@
         <v>80862.250366762659</v>
       </c>
       <c r="E100" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2005-Q3", annualized_gdp_million: 1637032, population_persons: 20244700, annualized_gdp_pc: 80862 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2005-Q3", annualized_gdp_million: 1637032, population_persons: 20244700},</v>
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.35">
@@ -4811,8 +4804,8 @@
         <v>81269.231716022943</v>
       </c>
       <c r="E101" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2005-Q4", annualized_gdp_million: 1650700, population_persons: 20311500, annualized_gdp_pc: 81269 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2005-Q4", annualized_gdp_million: 1650700, population_persons: 20311500},</v>
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.35">
@@ -4833,8 +4826,8 @@
         <v>80977.542025973002</v>
       </c>
       <c r="E102" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2006-Q1", annualized_gdp_million: 1651788, population_persons: 20398100, annualized_gdp_pc: 80978 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2006-Q1", annualized_gdp_million: 1651788, population_persons: 20398100},</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.35">
@@ -4855,8 +4848,8 @@
         <v>80965.820742261989</v>
       </c>
       <c r="E103" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2006-Q2", annualized_gdp_million: 1655832, population_persons: 20451000, annualized_gdp_pc: 80966 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2006-Q2", annualized_gdp_million: 1655832, population_persons: 20451000},</v>
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.35">
@@ -4877,8 +4870,8 @@
         <v>81827.059287421565</v>
       </c>
       <c r="E104" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2006-Q3", annualized_gdp_million: 1680916, population_persons: 20542300, annualized_gdp_pc: 81827 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2006-Q3", annualized_gdp_million: 1680916, population_persons: 20542300},</v>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.35">
@@ -4899,8 +4892,8 @@
         <v>82516.058659556424</v>
       </c>
       <c r="E105" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2006-Q4", annualized_gdp_million: 1702100, population_persons: 20627500, annualized_gdp_pc: 82516 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2006-Q4", annualized_gdp_million: 1702100, population_persons: 20627500},</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.35">
@@ -4921,8 +4914,8 @@
         <v>83171.220857357737</v>
       </c>
       <c r="E106" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2007-Q1", annualized_gdp_million: 1725204, population_persons: 20742800, annualized_gdp_pc: 83171 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2007-Q1", annualized_gdp_million: 1725204, population_persons: 20742800},</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.35">
@@ -4943,8 +4936,8 @@
         <v>83350.93817818664</v>
       </c>
       <c r="E107" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2007-Q2", annualized_gdp_million: 1736000, population_persons: 20827600, annualized_gdp_pc: 83351 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2007-Q2", annualized_gdp_million: 1736000, population_persons: 20827600},</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.35">
@@ -4965,8 +4958,8 @@
         <v>83959.816862771331</v>
       </c>
       <c r="E108" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2007-Q3", annualized_gdp_million: 1756792, population_persons: 20924200, annualized_gdp_pc: 83960 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2007-Q3", annualized_gdp_million: 1756792, population_persons: 20924200},</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.35">
@@ -4987,8 +4980,8 @@
         <v>83886.544125694112</v>
       </c>
       <c r="E109" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2007-Q4", annualized_gdp_million: 1762968, population_persons: 21016100, annualized_gdp_pc: 83887 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2007-Q4", annualized_gdp_million: 1762968, population_persons: 21016100},</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.35">
@@ -5009,8 +5002,8 @@
         <v>84265.942909560312</v>
       </c>
       <c r="E110" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2008-Q1", annualized_gdp_million: 1782132, population_persons: 21148900, annualized_gdp_pc: 84266 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2008-Q1", annualized_gdp_million: 1782132, population_persons: 21148900},</v>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.35">
@@ -5031,8 +5024,8 @@
         <v>84133.802684336348</v>
       </c>
       <c r="E111" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2008-Q2", annualized_gdp_million: 1787776, population_persons: 21249200, annualized_gdp_pc: 84134 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2008-Q2", annualized_gdp_million: 1787776, population_persons: 21249200},</v>
       </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.35">
@@ -5053,8 +5046,8 @@
         <v>84240.007488533185</v>
       </c>
       <c r="E112" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2008-Q3", annualized_gdp_million: 1799872, population_persons: 21366000, annualized_gdp_pc: 84240 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2008-Q3", annualized_gdp_million: 1799872, population_persons: 21366000},</v>
       </c>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.35">
@@ -5075,8 +5068,8 @@
         <v>83458.809067034221</v>
       </c>
       <c r="E113" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2008-Q4", annualized_gdp_million: 1792328, population_persons: 21475600, annualized_gdp_pc: 83459 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2008-Q4", annualized_gdp_million: 1792328, population_persons: 21475600},</v>
       </c>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.35">
@@ -5097,8 +5090,8 @@
         <v>83792.479295610989</v>
       </c>
       <c r="E114" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2009-Q1", annualized_gdp_million: 1810060, population_persons: 21601700, annualized_gdp_pc: 83792 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2009-Q1", annualized_gdp_million: 1810060, population_persons: 21601700},</v>
       </c>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.35">
@@ -5119,8 +5112,8 @@
         <v>83976.451822586518</v>
       </c>
       <c r="E115" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2009-Q2", annualized_gdp_million: 1821592, population_persons: 21691700, annualized_gdp_pc: 83976 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2009-Q2", annualized_gdp_million: 1821592, population_persons: 21691700},</v>
       </c>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.35">
@@ -5141,8 +5134,8 @@
         <v>83906.168963792166</v>
       </c>
       <c r="E116" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2009-Q3", annualized_gdp_million: 1828156, population_persons: 21788100, annualized_gdp_pc: 83906 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2009-Q3", annualized_gdp_million: 1828156, population_persons: 21788100},</v>
       </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.35">
@@ -5163,8 +5156,8 @@
         <v>84284.721205912487</v>
       </c>
       <c r="E117" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2009-Q4", annualized_gdp_million: 1842936, population_persons: 21865600, annualized_gdp_pc: 84285 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2009-Q4", annualized_gdp_million: 1842936, population_persons: 21865600},</v>
       </c>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.35">
@@ -5181,12 +5174,12 @@
         <v>21964100</v>
       </c>
       <c r="D118" s="16">
-        <f t="shared" ref="D118:D146" si="6">(B118*1000000)/C118</f>
+        <f t="shared" ref="D118:D146" si="5">(B118*1000000)/C118</f>
         <v>84272.608483844087</v>
       </c>
       <c r="E118" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2010-Q1", annualized_gdp_million: 1850972, population_persons: 21964100, annualized_gdp_pc: 84273 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2010-Q1", annualized_gdp_million: 1850972, population_persons: 21964100},</v>
       </c>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.35">
@@ -5203,12 +5196,12 @@
         <v>22031800</v>
       </c>
       <c r="D119" s="16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>84521.101317186971</v>
       </c>
       <c r="E119" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2010-Q2", annualized_gdp_million: 1862152, population_persons: 22031800, annualized_gdp_pc: 84521 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2010-Q2", annualized_gdp_million: 1862152, population_persons: 22031800},</v>
       </c>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.35">
@@ -5225,12 +5218,12 @@
         <v>22104400</v>
       </c>
       <c r="D120" s="16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>84846.817828124724</v>
       </c>
       <c r="E120" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2010-Q3", annualized_gdp_million: 1875488, population_persons: 22104400, annualized_gdp_pc: 84847 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2010-Q3", annualized_gdp_million: 1875488, population_persons: 22104400},</v>
       </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.35">
@@ -5247,12 +5240,12 @@
         <v>22172500</v>
       </c>
       <c r="D121" s="16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>85277.167662645166</v>
       </c>
       <c r="E121" t="str">
-        <f t="shared" si="5"/>
-        <v>{ quarter: "2010-Q4", annualized_gdp_million: 1890808, population_persons: 22172500, annualized_gdp_pc: 85277 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2010-Q4", annualized_gdp_million: 1890808, population_persons: 22172500},</v>
       </c>
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.35">
@@ -5269,15 +5262,12 @@
         <v>22268800</v>
       </c>
       <c r="D122" s="16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>84724.277913493323</v>
       </c>
       <c r="E122" t="str">
-        <f>"{ quarter: """ &amp; A122 &amp; """, " &amp;
- "annualized_gdp_million: " &amp; TEXT(B122,"0") &amp; ", " &amp;
- "population_persons: " &amp; TEXT(C122,"0") &amp; ", " &amp;
- "annualized_gdp_pc: " &amp; TEXT(D122,"0") &amp; " },"</f>
-        <v>{ quarter: "2011-Q1", annualized_gdp_million: 1886708, population_persons: 22268800, annualized_gdp_pc: 84724 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2011-Q1", annualized_gdp_million: 1886708, population_persons: 22268800},</v>
       </c>
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.35">
@@ -5294,15 +5284,12 @@
         <v>22340000</v>
       </c>
       <c r="D123" s="16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>85450.134288272151</v>
       </c>
       <c r="E123" t="str">
-        <f t="shared" ref="E123:E168" si="7">"{ quarter: """ &amp; A123 &amp; """, " &amp;
- "annualized_gdp_million: " &amp; TEXT(B123,"0") &amp; ", " &amp;
- "population_persons: " &amp; TEXT(C123,"0") &amp; ", " &amp;
- "annualized_gdp_pc: " &amp; TEXT(D123,"0") &amp; " },"</f>
-        <v>{ quarter: "2011-Q2", annualized_gdp_million: 1908956, population_persons: 22340000, annualized_gdp_pc: 85450 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2011-Q2", annualized_gdp_million: 1908956, population_persons: 22340000},</v>
       </c>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.35">
@@ -5319,12 +5306,12 @@
         <v>22432800</v>
       </c>
       <c r="D124" s="16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>86280.80310973218</v>
       </c>
       <c r="E124" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2011-Q3", annualized_gdp_million: 1935520, population_persons: 22432800, annualized_gdp_pc: 86281 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2011-Q3", annualized_gdp_million: 1935520, population_persons: 22432800},</v>
       </c>
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.35">
@@ -5341,12 +5328,12 @@
         <v>22522200</v>
       </c>
       <c r="D125" s="16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>86873.040821944567</v>
       </c>
       <c r="E125" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2011-Q4", annualized_gdp_million: 1956572, population_persons: 22522200, annualized_gdp_pc: 86873 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2011-Q4", annualized_gdp_million: 1956572, population_persons: 22522200},</v>
       </c>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.35">
@@ -5363,12 +5350,12 @@
         <v>22640900</v>
       </c>
       <c r="D126" s="16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>87280.629303605427</v>
       </c>
       <c r="E126" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2012-Q1", annualized_gdp_million: 1976112, population_persons: 22640900, annualized_gdp_pc: 87281 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2012-Q1", annualized_gdp_million: 1976112, population_persons: 22640900},</v>
       </c>
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.35">
@@ -5385,12 +5372,12 @@
         <v>22733500</v>
       </c>
       <c r="D127" s="16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>87533.199903226516</v>
       </c>
       <c r="E127" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2012-Q2", annualized_gdp_million: 1989936, population_persons: 22733500, annualized_gdp_pc: 87533 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2012-Q2", annualized_gdp_million: 1989936, population_persons: 22733500},</v>
       </c>
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.35">
@@ -5407,12 +5394,12 @@
         <v>22833900</v>
       </c>
       <c r="D128" s="16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>87694.699547602475</v>
       </c>
       <c r="E128" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2012-Q3", annualized_gdp_million: 2002412, population_persons: 22833900, annualized_gdp_pc: 87695 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2012-Q3", annualized_gdp_million: 2002412, population_persons: 22833900},</v>
       </c>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.35">
@@ -5429,12 +5416,12 @@
         <v>22928000</v>
       </c>
       <c r="D129" s="16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>87690.858339148646</v>
       </c>
       <c r="E129" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2012-Q4", annualized_gdp_million: 2010576, population_persons: 22928000, annualized_gdp_pc: 87691 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2012-Q4", annualized_gdp_million: 2010576, population_persons: 22928000},</v>
       </c>
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.35">
@@ -5451,12 +5438,12 @@
         <v>23043000</v>
       </c>
       <c r="D130" s="16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>87708.544894327992</v>
       </c>
       <c r="E130" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2013-Q1", annualized_gdp_million: 2021068, population_persons: 23043000, annualized_gdp_pc: 87709 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2013-Q1", annualized_gdp_million: 2021068, population_persons: 23043000},</v>
       </c>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.35">
@@ -5473,12 +5460,12 @@
         <v>23128100</v>
       </c>
       <c r="D131" s="16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>87710.274514551566</v>
       </c>
       <c r="E131" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2013-Q2", annualized_gdp_million: 2028572, population_persons: 23128100, annualized_gdp_pc: 87710 },</v>
+        <f t="shared" si="3"/>
+        <v>{ quarter: "2013-Q2", annualized_gdp_million: 2028572, population_persons: 23128100},</v>
       </c>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.35">
@@ -5495,12 +5482,14 @@
         <v>23220200</v>
       </c>
       <c r="D132" s="16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>88073.660002928489</v>
       </c>
       <c r="E132" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2013-Q3", annualized_gdp_million: 2045088, population_persons: 23220200, annualized_gdp_pc: 88074 },</v>
+        <f t="shared" ref="E132:E177" si="6">"{ quarter: """ &amp; A132 &amp; """, " &amp;
+ "annualized_gdp_million: " &amp; TEXT(B132,"0") &amp; ", " &amp;
+ "population_persons: " &amp; TEXT(C132,"0") &amp; "},"</f>
+        <v>{ quarter: "2013-Q3", annualized_gdp_million: 2045088, population_persons: 23220200},</v>
       </c>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.35">
@@ -5517,12 +5506,12 @@
         <v>23297800</v>
       </c>
       <c r="D133" s="16">
+        <f t="shared" si="5"/>
+        <v>88478.740481933914</v>
+      </c>
+      <c r="E133" t="str">
         <f t="shared" si="6"/>
-        <v>88478.740481933914</v>
-      </c>
-      <c r="E133" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2013-Q4", annualized_gdp_million: 2061360, population_persons: 23297800, annualized_gdp_pc: 88479 },</v>
+        <v>{ quarter: "2013-Q4", annualized_gdp_million: 2061360, population_persons: 23297800},</v>
       </c>
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.35">
@@ -5539,12 +5528,12 @@
         <v>23406200</v>
       </c>
       <c r="D134" s="16">
+        <f t="shared" si="5"/>
+        <v>88758.704958515271</v>
+      </c>
+      <c r="E134" t="str">
         <f t="shared" si="6"/>
-        <v>88758.704958515271</v>
-      </c>
-      <c r="E134" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2014-Q1", annualized_gdp_million: 2077504, population_persons: 23406200, annualized_gdp_pc: 88759 },</v>
+        <v>{ quarter: "2014-Q1", annualized_gdp_million: 2077504, population_persons: 23406200},</v>
       </c>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.35">
@@ -5561,12 +5550,12 @@
         <v>23475700</v>
       </c>
       <c r="D135" s="16">
+        <f t="shared" si="5"/>
+        <v>88939.626933382184</v>
+      </c>
+      <c r="E135" t="str">
         <f t="shared" si="6"/>
-        <v>88939.626933382184</v>
-      </c>
-      <c r="E135" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2014-Q2", annualized_gdp_million: 2087920, population_persons: 23475700, annualized_gdp_pc: 88940 },</v>
+        <v>{ quarter: "2014-Q2", annualized_gdp_million: 2087920, population_persons: 23475700},</v>
       </c>
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.35">
@@ -5583,12 +5572,12 @@
         <v>23562900</v>
       </c>
       <c r="D136" s="16">
+        <f t="shared" si="5"/>
+        <v>88967.487024092959</v>
+      </c>
+      <c r="E136" t="str">
         <f t="shared" si="6"/>
-        <v>88967.487024092959</v>
-      </c>
-      <c r="E136" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2014-Q3", annualized_gdp_million: 2096332, population_persons: 23562900, annualized_gdp_pc: 88967 },</v>
+        <v>{ quarter: "2014-Q3", annualized_gdp_million: 2096332, population_persons: 23562900},</v>
       </c>
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.35">
@@ -5605,12 +5594,12 @@
         <v>23640300</v>
       </c>
       <c r="D137" s="16">
+        <f t="shared" si="5"/>
+        <v>89013.421995490746</v>
+      </c>
+      <c r="E137" t="str">
         <f t="shared" si="6"/>
-        <v>89013.421995490746</v>
-      </c>
-      <c r="E137" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2014-Q4", annualized_gdp_million: 2104304, population_persons: 23640300, annualized_gdp_pc: 89013 },</v>
+        <v>{ quarter: "2014-Q4", annualized_gdp_million: 2104304, population_persons: 23640300},</v>
       </c>
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.35">
@@ -5627,12 +5616,12 @@
         <v>23745600</v>
       </c>
       <c r="D138" s="16">
+        <f t="shared" si="5"/>
+        <v>89490.768816117517</v>
+      </c>
+      <c r="E138" t="str">
         <f t="shared" si="6"/>
-        <v>89490.768816117517</v>
-      </c>
-      <c r="E138" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2015-Q1", annualized_gdp_million: 2125012, population_persons: 23745600, annualized_gdp_pc: 89491 },</v>
+        <v>{ quarter: "2015-Q1", annualized_gdp_million: 2125012, population_persons: 23745600},</v>
       </c>
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.35">
@@ -5649,12 +5638,12 @@
         <v>23816000</v>
       </c>
       <c r="D139" s="16">
+        <f t="shared" si="5"/>
+        <v>89326.167282499155</v>
+      </c>
+      <c r="E139" t="str">
         <f t="shared" si="6"/>
-        <v>89326.167282499155</v>
-      </c>
-      <c r="E139" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2015-Q2", annualized_gdp_million: 2127392, population_persons: 23816000, annualized_gdp_pc: 89326 },</v>
+        <v>{ quarter: "2015-Q2", annualized_gdp_million: 2127392, population_persons: 23816000},</v>
       </c>
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.35">
@@ -5671,12 +5660,12 @@
         <v>23904300</v>
       </c>
       <c r="D140" s="16">
+        <f t="shared" si="5"/>
+        <v>89857.975343348269</v>
+      </c>
+      <c r="E140" t="str">
         <f t="shared" si="6"/>
-        <v>89857.975343348269</v>
-      </c>
-      <c r="E140" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2015-Q3", annualized_gdp_million: 2147992, population_persons: 23904300, annualized_gdp_pc: 89858 },</v>
+        <v>{ quarter: "2015-Q3", annualized_gdp_million: 2147992, population_persons: 23904300},</v>
       </c>
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.35">
@@ -5693,12 +5682,12 @@
         <v>23984600</v>
       </c>
       <c r="D141" s="16">
+        <f t="shared" si="5"/>
+        <v>90118.159152122607</v>
+      </c>
+      <c r="E141" t="str">
         <f t="shared" si="6"/>
-        <v>90118.159152122607</v>
-      </c>
-      <c r="E141" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2015-Q4", annualized_gdp_million: 2161448, population_persons: 23984600, annualized_gdp_pc: 90118 },</v>
+        <v>{ quarter: "2015-Q4", annualized_gdp_million: 2161448, population_persons: 23984600},</v>
       </c>
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.35">
@@ -5715,12 +5704,12 @@
         <v>24103400</v>
       </c>
       <c r="D142" s="16">
+        <f t="shared" si="5"/>
+        <v>90503.248504360381</v>
+      </c>
+      <c r="E142" t="str">
         <f t="shared" si="6"/>
-        <v>90503.248504360381</v>
-      </c>
-      <c r="E142" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2016-Q1", annualized_gdp_million: 2181436, population_persons: 24103400, annualized_gdp_pc: 90503 },</v>
+        <v>{ quarter: "2016-Q1", annualized_gdp_million: 2181436, population_persons: 24103400},</v>
       </c>
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.35">
@@ -5737,12 +5726,12 @@
         <v>24190900</v>
       </c>
       <c r="D143" s="16">
+        <f t="shared" si="5"/>
+        <v>90753.795848852256</v>
+      </c>
+      <c r="E143" t="str">
         <f t="shared" si="6"/>
-        <v>90753.795848852256</v>
-      </c>
-      <c r="E143" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2016-Q2", annualized_gdp_million: 2195416, population_persons: 24190900, annualized_gdp_pc: 90754 },</v>
+        <v>{ quarter: "2016-Q2", annualized_gdp_million: 2195416, population_persons: 24190900},</v>
       </c>
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.35">
@@ -5759,12 +5748,12 @@
         <v>24297500</v>
       </c>
       <c r="D144" s="16">
+        <f t="shared" si="5"/>
+        <v>90344.274102273892</v>
+      </c>
+      <c r="E144" t="str">
         <f t="shared" si="6"/>
-        <v>90344.274102273892</v>
-      </c>
-      <c r="E144" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2016-Q3", annualized_gdp_million: 2195140, population_persons: 24297500, annualized_gdp_pc: 90344 },</v>
+        <v>{ quarter: "2016-Q3", annualized_gdp_million: 2195140, population_persons: 24297500},</v>
       </c>
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.35">
@@ -5781,12 +5770,12 @@
         <v>24385100</v>
       </c>
       <c r="D145" s="16">
+        <f t="shared" si="5"/>
+        <v>91060.852733841573</v>
+      </c>
+      <c r="E145" t="str">
         <f t="shared" si="6"/>
-        <v>91060.852733841573</v>
-      </c>
-      <c r="E145" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2016-Q4", annualized_gdp_million: 2220528, population_persons: 24385100, annualized_gdp_pc: 91061 },</v>
+        <v>{ quarter: "2016-Q4", annualized_gdp_million: 2220528, population_persons: 24385100},</v>
       </c>
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.35">
@@ -5803,12 +5792,12 @@
         <v>24511400</v>
       </c>
       <c r="D146" s="16">
+        <f t="shared" si="5"/>
+        <v>90877.714043261498</v>
+      </c>
+      <c r="E146" t="str">
         <f t="shared" si="6"/>
-        <v>90877.714043261498</v>
-      </c>
-      <c r="E146" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2017-Q1", annualized_gdp_million: 2227540, population_persons: 24511400, annualized_gdp_pc: 90878 },</v>
+        <v>{ quarter: "2017-Q1", annualized_gdp_million: 2227540, population_persons: 24511400},</v>
       </c>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.35">
@@ -5829,8 +5818,8 @@
         <v>91128.876166001151</v>
       </c>
       <c r="E147" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2017-Q2", annualized_gdp_million: 2241096, population_persons: 24592600, annualized_gdp_pc: 91129 },</v>
+        <f t="shared" si="6"/>
+        <v>{ quarter: "2017-Q2", annualized_gdp_million: 2241096, population_persons: 24592600},</v>
       </c>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.35">
@@ -5847,12 +5836,12 @@
         <v>24690100</v>
       </c>
       <c r="D148" s="16">
-        <f t="shared" ref="D148:D172" si="8">(B148*1000000)/C148</f>
+        <f t="shared" ref="D148:D172" si="7">(B148*1000000)/C148</f>
         <v>91605.947323016109</v>
       </c>
       <c r="E148" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2017-Q3", annualized_gdp_million: 2261760, population_persons: 24690100, annualized_gdp_pc: 91606 },</v>
+        <f t="shared" si="6"/>
+        <v>{ quarter: "2017-Q3", annualized_gdp_million: 2261760, population_persons: 24690100},</v>
       </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.35">
@@ -5869,12 +5858,12 @@
         <v>24759000</v>
       </c>
       <c r="D149" s="16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>91739.407892079646</v>
       </c>
       <c r="E149" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2017-Q4", annualized_gdp_million: 2271376, population_persons: 24759000, annualized_gdp_pc: 91739 },</v>
+        <f t="shared" si="6"/>
+        <v>{ quarter: "2017-Q4", annualized_gdp_million: 2271376, population_persons: 24759000},</v>
       </c>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.35">
@@ -5891,12 +5880,12 @@
         <v>24881800</v>
       </c>
       <c r="D150" s="16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>92235.127683688479</v>
       </c>
       <c r="E150" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2018-Q1", annualized_gdp_million: 2294976, population_persons: 24881800, annualized_gdp_pc: 92235 },</v>
+        <f t="shared" si="6"/>
+        <v>{ quarter: "2018-Q1", annualized_gdp_million: 2294976, population_persons: 24881800},</v>
       </c>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.35">
@@ -5913,12 +5902,12 @@
         <v>24963300</v>
       </c>
       <c r="D151" s="16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>92612.915760336167</v>
       </c>
       <c r="E151" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2018-Q2", annualized_gdp_million: 2311924, population_persons: 24963300, annualized_gdp_pc: 92613 },</v>
+        <f t="shared" si="6"/>
+        <v>{ quarter: "2018-Q2", annualized_gdp_million: 2311924, population_persons: 24963300},</v>
       </c>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.35">
@@ -5935,12 +5924,12 @@
         <v>25067400</v>
       </c>
       <c r="D152" s="16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>92562.132490804797</v>
       </c>
       <c r="E152" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2018-Q3", annualized_gdp_million: 2320292, population_persons: 25067400, annualized_gdp_pc: 92562 },</v>
+        <f t="shared" si="6"/>
+        <v>{ quarter: "2018-Q3", annualized_gdp_million: 2320292, population_persons: 25067400},</v>
       </c>
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.35">
@@ -5957,12 +5946,12 @@
         <v>25146100</v>
       </c>
       <c r="D153" s="16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>92493.706777591753</v>
       </c>
       <c r="E153" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2018-Q4", annualized_gdp_million: 2325856, population_persons: 25146100, annualized_gdp_pc: 92494 },</v>
+        <f t="shared" si="6"/>
+        <v>{ quarter: "2018-Q4", annualized_gdp_million: 2325856, population_persons: 25146100},</v>
       </c>
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.35">
@@ -5979,12 +5968,12 @@
         <v>25264900</v>
       </c>
       <c r="D154" s="16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>92728.805576115483</v>
       </c>
       <c r="E154" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2019-Q1", annualized_gdp_million: 2342784, population_persons: 25264900, annualized_gdp_pc: 92729 },</v>
+        <f t="shared" si="6"/>
+        <v>{ quarter: "2019-Q1", annualized_gdp_million: 2342784, population_persons: 25264900},</v>
       </c>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.35">
@@ -6001,12 +5990,12 @@
         <v>25334800</v>
       </c>
       <c r="D155" s="16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>92741.367605033389</v>
       </c>
       <c r="E155" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2019-Q2", annualized_gdp_million: 2349584, population_persons: 25334800, annualized_gdp_pc: 92741 },</v>
+        <f t="shared" si="6"/>
+        <v>{ quarter: "2019-Q2", annualized_gdp_million: 2349584, population_persons: 25334800},</v>
       </c>
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.35">
@@ -6023,12 +6012,12 @@
         <v>25438100</v>
       </c>
       <c r="D156" s="16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>92882.408670458884</v>
       </c>
       <c r="E156" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2019-Q3", annualized_gdp_million: 2362752, population_persons: 25438100, annualized_gdp_pc: 92882 },</v>
+        <f t="shared" si="6"/>
+        <v>{ quarter: "2019-Q3", annualized_gdp_million: 2362752, population_persons: 25438100},</v>
       </c>
     </row>
     <row r="157" spans="1:5" x14ac:dyDescent="0.35">
@@ -6045,12 +6034,12 @@
         <v>25520500</v>
       </c>
       <c r="D157" s="16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>93142.532473893531</v>
       </c>
       <c r="E157" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2019-Q4", annualized_gdp_million: 2377044, population_persons: 25520500, annualized_gdp_pc: 93143 },</v>
+        <f t="shared" si="6"/>
+        <v>{ quarter: "2019-Q4", annualized_gdp_million: 2377044, population_persons: 25520500},</v>
       </c>
     </row>
     <row r="158" spans="1:5" x14ac:dyDescent="0.35">
@@ -6067,12 +6056,12 @@
         <v>25627900</v>
       </c>
       <c r="D158" s="16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>92629.829209572374</v>
       </c>
       <c r="E158" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2020-Q1", annualized_gdp_million: 2373908, population_persons: 25627900, annualized_gdp_pc: 92630 },</v>
+        <f t="shared" si="6"/>
+        <v>{ quarter: "2020-Q1", annualized_gdp_million: 2373908, population_persons: 25627900},</v>
       </c>
     </row>
     <row r="159" spans="1:5" x14ac:dyDescent="0.35">
@@ -6089,12 +6078,12 @@
         <v>25649200</v>
       </c>
       <c r="D159" s="16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>86304.602092852801</v>
       </c>
       <c r="E159" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2020-Q2", annualized_gdp_million: 2213644, population_persons: 25649200, annualized_gdp_pc: 86305 },</v>
+        <f t="shared" si="6"/>
+        <v>{ quarter: "2020-Q2", annualized_gdp_million: 2213644, population_persons: 25649200},</v>
       </c>
     </row>
     <row r="160" spans="1:5" x14ac:dyDescent="0.35">
@@ -6111,12 +6100,12 @@
         <v>25633300</v>
       </c>
       <c r="D160" s="16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>89376.241061431807</v>
       </c>
       <c r="E160" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2020-Q3", annualized_gdp_million: 2291008, population_persons: 25633300, annualized_gdp_pc: 89376 },</v>
+        <f t="shared" si="6"/>
+        <v>{ quarter: "2020-Q3", annualized_gdp_million: 2291008, population_persons: 25633300},</v>
       </c>
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.35">
@@ -6133,12 +6122,12 @@
         <v>25630700</v>
       </c>
       <c r="D161" s="16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>92441.798312180312</v>
       </c>
       <c r="E161" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2020-Q4", annualized_gdp_million: 2369348, population_persons: 25630700, annualized_gdp_pc: 92442 },</v>
+        <f t="shared" si="6"/>
+        <v>{ quarter: "2020-Q4", annualized_gdp_million: 2369348, population_persons: 25630700},</v>
       </c>
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.35">
@@ -6155,12 +6144,12 @@
         <v>25653000</v>
       </c>
       <c r="D162" s="16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>94431.996257747625</v>
       </c>
       <c r="E162" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2021-Q1", annualized_gdp_million: 2422464, population_persons: 25653000, annualized_gdp_pc: 94432 },</v>
+        <f t="shared" si="6"/>
+        <v>{ quarter: "2021-Q1", annualized_gdp_million: 2422464, population_persons: 25653000},</v>
       </c>
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.35">
@@ -6177,12 +6166,12 @@
         <v>25685400</v>
       </c>
       <c r="D163" s="16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>95051.819321482239</v>
       </c>
       <c r="E163" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2021-Q2", annualized_gdp_million: 2441444, population_persons: 25685400, annualized_gdp_pc: 95052 },</v>
+        <f t="shared" si="6"/>
+        <v>{ quarter: "2021-Q2", annualized_gdp_million: 2441444, population_persons: 25685400},</v>
       </c>
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.35">
@@ -6199,12 +6188,12 @@
         <v>25704800</v>
       </c>
       <c r="D164" s="16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>93369.954249789924</v>
       </c>
       <c r="E164" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2021-Q3", annualized_gdp_million: 2400056, population_persons: 25704800, annualized_gdp_pc: 93370 },</v>
+        <f t="shared" si="6"/>
+        <v>{ quarter: "2021-Q3", annualized_gdp_million: 2400056, population_persons: 25704800},</v>
       </c>
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.35">
@@ -6221,12 +6210,12 @@
         <v>25773800</v>
       </c>
       <c r="D165" s="16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>96415.740015054049</v>
       </c>
       <c r="E165" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2021-Q4", annualized_gdp_million: 2485000, population_persons: 25773800, annualized_gdp_pc: 96416 },</v>
+        <f t="shared" si="6"/>
+        <v>{ quarter: "2021-Q4", annualized_gdp_million: 2485000, population_persons: 25773800},</v>
       </c>
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.35">
@@ -6243,12 +6232,12 @@
         <v>25913000</v>
       </c>
       <c r="D166" s="16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>96839.578589896963</v>
       </c>
       <c r="E166" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2022-Q1", annualized_gdp_million: 2509404, population_persons: 25913000, annualized_gdp_pc: 96840 },</v>
+        <f t="shared" si="6"/>
+        <v>{ quarter: "2022-Q1", annualized_gdp_million: 2509404, population_persons: 25913000},</v>
       </c>
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.35">
@@ -6265,12 +6254,12 @@
         <v>26018700</v>
       </c>
       <c r="D167" s="16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>97385.95702321791</v>
       </c>
       <c r="E167" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2022-Q2", annualized_gdp_million: 2533856, population_persons: 26018700, annualized_gdp_pc: 97386 },</v>
+        <f t="shared" si="6"/>
+        <v>{ quarter: "2022-Q2", annualized_gdp_million: 2533856, population_persons: 26018700},</v>
       </c>
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.35">
@@ -6287,12 +6276,12 @@
         <v>26169300</v>
       </c>
       <c r="D168" s="16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>97271.382879939469</v>
       </c>
       <c r="E168" t="str">
-        <f t="shared" si="7"/>
-        <v>{ quarter: "2022-Q3", annualized_gdp_million: 2545524, population_persons: 26169300, annualized_gdp_pc: 97271 },</v>
+        <f t="shared" si="6"/>
+        <v>{ quarter: "2022-Q3", annualized_gdp_million: 2545524, population_persons: 26169300},</v>
       </c>
     </row>
     <row r="169" spans="1:5" x14ac:dyDescent="0.35">
@@ -6309,15 +6298,12 @@
         <v>26320300</v>
       </c>
       <c r="D169" s="16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>97377.46150309837</v>
       </c>
       <c r="E169" t="str">
-        <f>"{ quarter: """ &amp; A169 &amp; """, " &amp;
- "annualized_gdp_million: " &amp; TEXT(B169,"0") &amp; ", " &amp;
- "population_persons: " &amp; TEXT(C169,"0") &amp; ", " &amp;
- "annualized_gdp_pc: " &amp; TEXT(D169,"0") &amp; " },"</f>
-        <v>{ quarter: "2022-Q4", annualized_gdp_million: 2563004, population_persons: 26320300, annualized_gdp_pc: 97377 },</v>
+        <f t="shared" si="6"/>
+        <v>{ quarter: "2022-Q4", annualized_gdp_million: 2563004, population_persons: 26320300},</v>
       </c>
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.35">
@@ -6334,15 +6320,12 @@
         <v>26514300</v>
       </c>
       <c r="D170" s="16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>97158.288169025778</v>
       </c>
       <c r="E170" t="str">
-        <f t="shared" ref="E170:E177" si="9">"{ quarter: """ &amp; A170 &amp; """, " &amp;
- "annualized_gdp_million: " &amp; TEXT(B170,"0") &amp; ", " &amp;
- "population_persons: " &amp; TEXT(C170,"0") &amp; ", " &amp;
- "annualized_gdp_pc: " &amp; TEXT(D170,"0") &amp; " },"</f>
-        <v>{ quarter: "2023-Q1", annualized_gdp_million: 2576084, population_persons: 26514300, annualized_gdp_pc: 97158 },</v>
+        <f t="shared" si="6"/>
+        <v>{ quarter: "2023-Q1", annualized_gdp_million: 2576084, population_persons: 26514300},</v>
       </c>
     </row>
     <row r="171" spans="1:5" x14ac:dyDescent="0.35">
@@ -6359,12 +6342,12 @@
         <v>26659900</v>
       </c>
       <c r="D171" s="16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>96978.60832186167</v>
       </c>
       <c r="E171" t="str">
-        <f t="shared" si="9"/>
-        <v>{ quarter: "2023-Q2", annualized_gdp_million: 2585440, population_persons: 26659900, annualized_gdp_pc: 96979 },</v>
+        <f t="shared" si="6"/>
+        <v>{ quarter: "2023-Q2", annualized_gdp_million: 2585440, population_persons: 26659900},</v>
       </c>
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.35">
@@ -6381,12 +6364,12 @@
         <v>26832500</v>
       </c>
       <c r="D172" s="16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>96837.044628715172</v>
       </c>
       <c r="E172" t="str">
-        <f t="shared" si="9"/>
-        <v>{ quarter: "2023-Q3", annualized_gdp_million: 2598380, population_persons: 26832500, annualized_gdp_pc: 96837 },</v>
+        <f t="shared" si="6"/>
+        <v>{ quarter: "2023-Q3", annualized_gdp_million: 2598380, population_persons: 26832500},</v>
       </c>
     </row>
     <row r="173" spans="1:5" x14ac:dyDescent="0.35">
@@ -6407,8 +6390,8 @@
         <v>96520.380943900935</v>
       </c>
       <c r="E173" t="str">
-        <f t="shared" si="9"/>
-        <v>{ quarter: "2023-Q4", annualized_gdp_million: 2601620, population_persons: 26954100, annualized_gdp_pc: 96520 },</v>
+        <f t="shared" si="6"/>
+        <v>{ quarter: "2023-Q4", annualized_gdp_million: 2601620, population_persons: 26954100},</v>
       </c>
     </row>
     <row r="174" spans="1:5" x14ac:dyDescent="0.35">
@@ -6425,12 +6408,12 @@
         <v>27113700</v>
       </c>
       <c r="D174" s="16">
-        <f t="shared" ref="D174:D177" si="10">(B174*1000000)/C174</f>
+        <f t="shared" ref="D174:D177" si="8">(B174*1000000)/C174</f>
         <v>96105.658762913212</v>
       </c>
       <c r="E174" t="str">
-        <f t="shared" si="9"/>
-        <v>{ quarter: "2024-Q1", annualized_gdp_million: 2605780, population_persons: 27113700, annualized_gdp_pc: 96106 },</v>
+        <f t="shared" si="6"/>
+        <v>{ quarter: "2024-Q1", annualized_gdp_million: 2605780, population_persons: 27113700},</v>
       </c>
     </row>
     <row r="175" spans="1:5" x14ac:dyDescent="0.35">
@@ -6447,12 +6430,12 @@
         <v>27196800</v>
       </c>
       <c r="D175" s="16">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>95944.964113425114</v>
       </c>
       <c r="E175" t="str">
-        <f t="shared" si="9"/>
-        <v>{ quarter: "2024-Q2", annualized_gdp_million: 2609396, population_persons: 27196800, annualized_gdp_pc: 95945 },</v>
+        <f t="shared" si="6"/>
+        <v>{ quarter: "2024-Q2", annualized_gdp_million: 2609396, population_persons: 27196800},</v>
       </c>
     </row>
     <row r="176" spans="1:5" x14ac:dyDescent="0.35">
@@ -6469,12 +6452,12 @@
         <v>27308900</v>
       </c>
       <c r="D176" s="16">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>95871.748770547332</v>
       </c>
       <c r="E176" t="str">
-        <f t="shared" si="9"/>
-        <v>{ quarter: "2024-Q3", annualized_gdp_million: 2618152, population_persons: 27308900, annualized_gdp_pc: 95872 },</v>
+        <f t="shared" si="6"/>
+        <v>{ quarter: "2024-Q3", annualized_gdp_million: 2618152, population_persons: 27308900},</v>
       </c>
     </row>
     <row r="177" spans="1:5" x14ac:dyDescent="0.35">
@@ -6491,12 +6474,12 @@
         <v>27400000</v>
       </c>
       <c r="D177" s="16">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>96138.248175182482</v>
       </c>
       <c r="E177" t="str">
-        <f t="shared" si="9"/>
-        <v>{ quarter: "2024-Q4", annualized_gdp_million: 2634188, population_persons: 27400000, annualized_gdp_pc: 96138 },</v>
+        <f t="shared" si="6"/>
+        <v>{ quarter: "2024-Q4", annualized_gdp_million: 2634188, population_persons: 27400000},</v>
       </c>
     </row>
     <row r="178" spans="1:5" x14ac:dyDescent="0.35">

</xml_diff>